<commit_message>
Move relevant files to wsn management algorithms folder
</commit_message>
<xml_diff>
--- a/docs/Papers/graph_search_papers.xlsx
+++ b/docs/Papers/graph_search_papers.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roman\PycharmProjects\bachelorThesis\docs\Papers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E424C3A-A023-463F-BE8A-65A6754F26E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A944F1CA-8A9A-406A-94F2-CBFE6B2974C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-18120" yWindow="-120" windowWidth="18240" windowHeight="29040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
   <si>
     <t>Reference</t>
   </si>
@@ -70,6 +70,30 @@
   </si>
   <si>
     <t>Kemmerling, M., Lütticke, D., &amp; Schmitt, R. H. (2023). Beyond games: a systematic review of neural Monte Carlo tree search applications. arXiv preprint arXiv:2303.08060.</t>
+  </si>
+  <si>
+    <t>Lowerre, B., &amp; Reddy, R. (1976). The harpy speech recognition system: performance with large vocabularies. The Journal of the Acoustical Society of America, 60(S1), S10-S11.</t>
+  </si>
+  <si>
+    <t>Hart, P. E., Nilsson, N. J., &amp; Raphael, B. (1968). A formal basis for the heuristic determination of minimum cost paths. IEEE transactions on Systems Science and Cybernetics, 4(2), 100-107.</t>
+  </si>
+  <si>
+    <t>Kahn, A. B. (1962). Topological sorting of large networks. Communications of the ACM, 5(11), 558-562.</t>
+  </si>
+  <si>
+    <t>(Wikipedia)</t>
+  </si>
+  <si>
+    <t>Topological Sorting</t>
+  </si>
+  <si>
+    <t>Metropolis, N., &amp; Ulam, S. (1949). The monte carlo method. Journal of the American statistical association, 44(247), 335-341.</t>
+  </si>
+  <si>
+    <t>Abramson, Bruce (1987). The Expected-Outcome Model of Two-Player Games (PDF). Technical report, Department of Computer Science, Columbia University.</t>
+  </si>
+  <si>
+    <t>Brügmann, B. (1993). Monte carlo go (Vol. 44). Syracuse, NY: Technical report, Physics Department, Syracuse University.</t>
   </si>
 </sst>
 </file>
@@ -407,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="64.7109375" customWidth="1"/>
@@ -525,6 +549,48 @@
         <v>3</v>
       </c>
     </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{36DBE1DB-3259-441B-BD30-2D546F9F93C3}"/>
@@ -534,8 +600,14 @@
     <hyperlink ref="A6" r:id="rId5" xr:uid="{E63B2AAA-9080-4984-898B-2E7D8366410B}"/>
     <hyperlink ref="A7" r:id="rId6" xr:uid="{B79B7228-4711-4EFA-AE72-7DB30FCD43C7}"/>
     <hyperlink ref="A8" r:id="rId7" xr:uid="{9232E035-3D84-4DBA-B7B4-2E4D56586EFA}"/>
+    <hyperlink ref="A10" r:id="rId8" display="Topological sorting of large networks" xr:uid="{6C9DAD47-4E69-4A36-AE52-6FAAA35F4492}"/>
+    <hyperlink ref="A11" r:id="rId9" xr:uid="{DF6E468E-16D0-4555-88BE-06CE0547A829}"/>
+    <hyperlink ref="A9" r:id="rId10" xr:uid="{52D39CF1-64BB-4F47-82B6-F9D8D82B3553}"/>
+    <hyperlink ref="A12" r:id="rId11" xr:uid="{E135C97D-0DE7-4AEF-84E2-EF1EE752C453}"/>
+    <hyperlink ref="A13" r:id="rId12" display="http://academiccommons.columbia.edu/download/fedora_content/download/ac:142327/CONTENT/CUCS-315-87.pdf" xr:uid="{F26D8E9C-584A-41D6-8E91-3C179A55D47E}"/>
+    <hyperlink ref="A14" r:id="rId13" xr:uid="{2F0AFF6F-9B3D-4DAA-A5A1-15AE9D11F751}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId8"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>